<commit_message>
Gera pedidos de envio por filial e registra histórico para não repetir itens
- Arquivos de envio Pedido_COMPRE_MAIS_20260930_Maraba.xlsx e _Castanhal.xlsx
- historico_pedidos.csv com os 74 itens pedidos em 30/09/2026
- O script exclui dos próximos pedidos os produtos já pedidos nos últimos
  30 dias (por código interno ou EAN) e lista-os na aba "Já pedidos"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4bXq8zCEB9pvU5LeoWnau
</commit_message>
<xml_diff>
--- a/pedidos/Pedido_COMPRE_MAIS_20260930.xlsx
+++ b/pedidos/Pedido_COMPRE_MAIS_20260930.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Comparativo" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo'!$A$1:$B$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pedido'!$A$1:$S$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pedido Marabá'!$A$1:$S$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pedido Castanhal'!$A$1:$S$28</definedName>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -488,89 +488,99 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Itens no pedido</t>
+          <t xml:space="preserve">  - já pedidos nos últimos 30 dias (fora deste pedido)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Itens mais baratos mas sem estoque no CM</t>
+          <t>Itens no pedido</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Caixas no pedido</t>
+          <t>Itens mais baratos mas sem estoque no CM</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>894</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pedido Marabá — itens / valor (R$)</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>47 / 3965.03</t>
-        </is>
+          <t>Caixas no pedido</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>894</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Pedido Castanhal — itens / valor (R$)</t>
+          <t>Pedido Marabá — itens / valor (R$)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>27 / 2349.07</t>
+          <t>47 / 3965.03</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Valor do pedido Compre Mais (R$)</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>6314.1</v>
+          <t>Pedido Castanhal — itens / valor (R$)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>27 / 2349.07</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mesmas unidades pelo preço da última compra (R$)</t>
+          <t>Valor do pedido Compre Mais (R$)</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>7075.82</v>
+        <v>6314.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Mesmas unidades pelo preço da última compra (R$)</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>7075.82</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Economia (R$)</t>
         </is>
       </c>
-      <c r="B13" s="1" t="n">
+      <c r="B14" s="1" t="n">
         <v>761.72</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>